<commit_message>
Price tracker: run numbering + alerts screenshot
</commit_message>
<xml_diff>
--- a/price-tracker/output/price_report.xlsx
+++ b/price-tracker/output/price_report.xlsx
@@ -211,12 +211,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Chart data'!$A$2:$A$5</f>
+              <f>'Chart data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart data'!$B$2:$B$5</f>
+              <f>'Chart data'!$B$2:$B$6</f>
             </numRef>
           </val>
         </ser>
@@ -243,12 +243,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Chart data'!$A$2:$A$5</f>
+              <f>'Chart data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart data'!$C$2:$C$5</f>
+              <f>'Chart data'!$C$2:$C$6</f>
             </numRef>
           </val>
         </ser>
@@ -275,12 +275,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Chart data'!$A$2:$A$5</f>
+              <f>'Chart data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart data'!$D$2:$D$5</f>
+              <f>'Chart data'!$D$2:$D$6</f>
             </numRef>
           </val>
         </ser>
@@ -307,12 +307,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Chart data'!$A$2:$A$5</f>
+              <f>'Chart data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart data'!$E$2:$E$5</f>
+              <f>'Chart data'!$E$2:$E$6</f>
             </numRef>
           </val>
         </ser>
@@ -339,12 +339,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Chart data'!$A$2:$A$5</f>
+              <f>'Chart data'!$A$2:$A$6</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Chart data'!$F$2:$F$5</f>
+              <f>'Chart data'!$F$2:$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -784,16 +784,16 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
+        <v>83434</v>
+      </c>
+      <c r="D2" s="2" t="n">
         <v>83400</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>83372</v>
-      </c>
       <c r="E2" s="3" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.034</v>
+        <v>0.041</v>
       </c>
     </row>
     <row r="3">
@@ -808,16 +808,16 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
+        <v>2505.77</v>
+      </c>
+      <c r="D3" s="2" t="n">
         <v>2509.21</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>2509.56</v>
-      </c>
       <c r="E3" s="5" t="n">
-        <v>-0.3499999999999091</v>
+        <v>-3.440000000000055</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>-0.014</v>
+        <v>-0.137</v>
       </c>
     </row>
     <row r="4">
@@ -832,16 +832,16 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
+        <v>0.999193</v>
+      </c>
+      <c r="D4" s="2" t="n">
         <v>0.9993339999999999</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>0.999337</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>-3.000000000086267e-06</v>
-      </c>
-      <c r="F4" s="7" t="n">
-        <v>-0</v>
+      <c r="E4" s="5" t="n">
+        <v>-0.0001409999999999467</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>-0.014</v>
       </c>
     </row>
     <row r="5">
@@ -856,16 +856,16 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
+        <v>741.38</v>
+      </c>
+      <c r="D5" s="2" t="n">
         <v>741.79</v>
       </c>
-      <c r="D5" s="2" t="n">
-        <v>741.9400000000001</v>
-      </c>
       <c r="E5" s="5" t="n">
-        <v>-0.1500000000000909</v>
+        <v>-0.4099999999999682</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>-0.02</v>
+        <v>-0.055</v>
       </c>
     </row>
     <row r="6">
@@ -904,16 +904,16 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
+        <v>0.9996969999999999</v>
+      </c>
+      <c r="D7" s="2" t="n">
         <v>0.999779</v>
       </c>
-      <c r="D7" s="2" t="n">
-        <v>0.999764</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1.499999999998725e-05</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>0.002</v>
+      <c r="E7" s="5" t="n">
+        <v>-8.20000000000265e-05</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>-0.008</v>
       </c>
     </row>
     <row r="8">
@@ -928,16 +928,16 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
+        <v>107.09</v>
+      </c>
+      <c r="D8" s="2" t="n">
         <v>107.04</v>
       </c>
-      <c r="D8" s="2" t="n">
-        <v>107.05</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>-0.009999999999990905</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>-0.008999999999999999</v>
+      <c r="E8" s="3" t="n">
+        <v>0.04999999999999716</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.047</v>
       </c>
     </row>
     <row r="9">
@@ -952,16 +952,16 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
+        <v>0.332691</v>
+      </c>
+      <c r="D9" s="2" t="n">
         <v>0.327799</v>
       </c>
-      <c r="D9" s="2" t="n">
-        <v>0.328113</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>-0.000313999999999981</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>-0.096</v>
+      <c r="E9" s="3" t="n">
+        <v>0.004892000000000007</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>1.492</v>
       </c>
     </row>
     <row r="10">
@@ -976,16 +976,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1.03</v>
+        <v>1.026</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>1.03</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>0</v>
+      <c r="E10" s="5" t="n">
+        <v>-0.004000000000000004</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>-0.388</v>
       </c>
     </row>
     <row r="11">
@@ -1000,16 +1000,16 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
+        <v>1243.1</v>
+      </c>
+      <c r="D11" s="2" t="n">
         <v>1221.36</v>
       </c>
-      <c r="D11" s="2" t="n">
-        <v>1221.31</v>
-      </c>
       <c r="E11" s="3" t="n">
-        <v>0.04999999999995453</v>
+        <v>21.74000000000001</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.004</v>
+        <v>1.78</v>
       </c>
     </row>
     <row r="12">
@@ -1024,16 +1024,16 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
+        <v>81.38</v>
+      </c>
+      <c r="D12" s="2" t="n">
         <v>81.75</v>
       </c>
-      <c r="D12" s="2" t="n">
-        <v>81.70999999999999</v>
-      </c>
-      <c r="E12" s="3" t="n">
-        <v>0.04000000000000625</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0.049</v>
+      <c r="E12" s="5" t="n">
+        <v>-0.3700000000000045</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>-0.453</v>
       </c>
     </row>
     <row r="13">
@@ -1048,64 +1048,64 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
+        <v>0.08441800000000001</v>
+      </c>
+      <c r="D13" s="2" t="n">
         <v>0.084582</v>
       </c>
-      <c r="D13" s="2" t="n">
-        <v>0.08458599999999999</v>
-      </c>
       <c r="E13" s="5" t="n">
-        <v>-3.999999999990123e-06</v>
+        <v>-0.0001639999999999975</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>-0.005</v>
+        <v>-0.194</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>USDS</t>
+          <t>XMR</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>USDS</t>
+          <t>Monero</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1</v>
+        <v>554.8</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
+        <v>541.87</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>12.92999999999995</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>2.386</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>XMR</t>
+          <t>USDS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Monero</t>
+          <t>USDS</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>541.87</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>540.83</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>1.039999999999964</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0.192</v>
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1120,16 +1120,16 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="D16" s="2" t="n">
         <v>12.91</v>
       </c>
-      <c r="D16" s="2" t="n">
-        <v>12.92</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>-0.009999999999999787</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>-0.077</v>
+      <c r="E16" s="3" t="n">
+        <v>0.05000000000000071</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.387</v>
       </c>
     </row>
     <row r="17">
@@ -1144,16 +1144,16 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
+        <v>81.92</v>
+      </c>
+      <c r="D17" s="2" t="n">
         <v>81.86</v>
       </c>
-      <c r="D17" s="2" t="n">
-        <v>81.84</v>
-      </c>
       <c r="E17" s="3" t="n">
-        <v>0.01999999999999602</v>
+        <v>0.06000000000000227</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.024</v>
+        <v>0.073</v>
       </c>
     </row>
     <row r="18">
@@ -1168,16 +1168,16 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
+        <v>0.235175</v>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>0.237334</v>
       </c>
-      <c r="D18" s="2" t="n">
-        <v>0.237061</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>0.0002729999999999955</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>0.115</v>
+      <c r="E18" s="5" t="n">
+        <v>-0.002158999999999994</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>-0.91</v>
       </c>
     </row>
     <row r="19">
@@ -1192,16 +1192,16 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>8.91</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>8.91</v>
       </c>
-      <c r="E19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>0</v>
+      <c r="E19" s="3" t="n">
+        <v>0.0600000000000005</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>0.673</v>
       </c>
     </row>
     <row r="20">
@@ -1216,16 +1216,16 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
+        <v>0.00976058</v>
+      </c>
+      <c r="D20" s="2" t="n">
         <v>0.01001101</v>
       </c>
-      <c r="D20" s="2" t="n">
-        <v>0.0100204</v>
-      </c>
       <c r="E20" s="5" t="n">
-        <v>-9.389999999999746e-06</v>
+        <v>-0.0002504300000000011</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>-0.094</v>
+        <v>-2.502</v>
       </c>
     </row>
     <row r="21">
@@ -1240,16 +1240,16 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
+        <v>0.189428</v>
+      </c>
+      <c r="D21" s="2" t="n">
         <v>0.191389</v>
       </c>
-      <c r="D21" s="2" t="n">
-        <v>0.191502</v>
-      </c>
       <c r="E21" s="5" t="n">
-        <v>-0.000113000000000002</v>
+        <v>-0.001960999999999991</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>-0.059</v>
+        <v>-1.025</v>
       </c>
     </row>
   </sheetData>
@@ -1263,14 +1263,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1306,8 +1306,176 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TRX</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TRON</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.332691</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.327799</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.004892000000000007</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.492</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
+        <is>
+          <t>ZEC</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Zcash</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1243.1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1221.36</v>
+      </c>
+      <c r="E3" t="n">
+        <v>21.74000000000001</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.78</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>XMR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monero</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>554.8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>541.87</v>
+      </c>
+      <c r="E4" t="n">
+        <v>12.92999999999995</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2.386</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ADA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cardano</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.235175</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.237334</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.002158999999999994</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LEO</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LEO Token</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>8.970000000000001</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.0600000000000005</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.673</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>RAIN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rain</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.00976058</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.01001101</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-0.0002504300000000011</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-2.502</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>XLM</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Stellar</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.189428</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.191389</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-0.001960999999999991</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-1.025</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Moves of 0.5% or more since the previous run</t>
         </is>
@@ -1324,7 +1492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1455,6 +1623,28 @@
         <v>1.37</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:14:20</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>83434</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2505.77</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.999193</v>
+      </c>
+      <c r="E6" t="n">
+        <v>741.38</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.37</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1467,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1598,6 +1788,28 @@
         <v>100</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-14 14:14:20</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>100.138</v>
+      </c>
+      <c r="C6" t="n">
+        <v>99.923</v>
+      </c>
+      <c r="D6" t="n">
+        <v>99.983</v>
+      </c>
+      <c r="E6" t="n">
+        <v>99.949</v>
+      </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>